<commit_message>
initial testing of effect of modified assumptions on financial performance
</commit_message>
<xml_diff>
--- a/data/financial_projections.xlsx
+++ b/data/financial_projections.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebbi Kankondi\fleet_management\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B63E688B-751F-4FAB-A8CF-425A4397AC7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C129C8B-793F-46B1-A7A9-8058F06D5095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
@@ -822,16 +822,16 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1069,12 +1069,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1572,20 +1572,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
+      <c r="A1" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
     </row>
     <row r="2" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -4222,24 +4222,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
     </row>
     <row r="2" spans="1:19" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -8298,11 +8298,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
       <c r="D1" s="11"/>
       <c r="E1" s="11"/>
       <c r="F1" s="11"/>
@@ -14069,15 +14069,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="26" t="s">
         <v>123</v>
       </c>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
       <c r="I1" s="11"/>
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
@@ -19696,24 +19696,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
     </row>
     <row r="2" spans="1:6" ht="28.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="28"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="25"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">

</xml_diff>

<commit_message>
Generate new data files based on different simulation scenarios & minor change to guide. nks
</commit_message>
<xml_diff>
--- a/data/financial_projections.xlsx
+++ b/data/financial_projections.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebbi Kankondi\fleet_management\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0555EB08-F0B7-4CDA-BFD0-1B80EFB0F771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BEAC718-754F-471F-9C02-F161E0B69523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,12 +210,6 @@
   </si>
   <si>
     <t>N$ / car / month</t>
-  </si>
-  <si>
-    <t>Vehicle disposal trigger</t>
-  </si>
-  <si>
-    <t>car trigger for the disposal (with no disposal revenue) of all vehicles.</t>
   </si>
   <si>
     <t>Procurement lead time</t>
@@ -599,6 +593,12 @@
   <si>
     <t xml:space="preserve">For client upkeep. Part of offset (used to offset operating profit for contracts 
 extended beyond 15months) funds accumulated paid as subsistence. </t>
+  </si>
+  <si>
+    <t>Contract length</t>
+  </si>
+  <si>
+    <t>Client contract length that doubles as trigger for the disposal (with no disposal revenue) of all vehicles.</t>
   </si>
 </sst>
 </file>
@@ -1125,35 +1125,35 @@
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>148</v>
       </c>
       <c r="B6" s="18">
         <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>23</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B7" s="4">
         <v>3</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B8" s="3">
         <v>13000</v>
@@ -1162,12 +1162,12 @@
         <v>21</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B9" s="3">
         <v>290</v>
@@ -1176,12 +1176,12 @@
         <v>21</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B10" s="3">
         <v>240</v>
@@ -1193,7 +1193,7 @@
     </row>
     <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B11" s="3">
         <v>0</v>
@@ -1202,12 +1202,12 @@
         <v>21</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B12" s="19">
         <v>500</v>
@@ -1216,12 +1216,12 @@
         <v>21</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B13" s="19">
         <v>0</v>
@@ -1230,12 +1230,12 @@
         <v>21</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B14" s="19">
         <v>970</v>
@@ -1244,12 +1244,12 @@
         <v>21</v>
       </c>
       <c r="D14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B15" s="19">
         <f>SUM(B8:B14)</f>
@@ -1259,12 +1259,12 @@
         <v>21</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B16" s="19">
         <f>B5-B15</f>
@@ -1274,12 +1274,12 @@
         <v>21</v>
       </c>
       <c r="D16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B17" s="19">
         <v>3000</v>
@@ -1288,12 +1288,12 @@
         <v>21</v>
       </c>
       <c r="D17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B18" s="19">
         <f>B15+B17</f>
@@ -1303,12 +1303,12 @@
         <v>21</v>
       </c>
       <c r="D18" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B19" s="19">
         <f>B5-B18</f>
@@ -1318,210 +1318,210 @@
         <v>21</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B20" s="4">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B21" s="5">
         <v>0.32</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B22" s="9">
         <v>250000</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B23" s="3">
         <v>250000</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B24" s="4">
         <v>5</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B25" s="20">
         <f>-PMT(B32,B31,B23)</f>
         <v>5768.1018465472143</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B26" s="10">
         <v>0.1</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B27" s="3">
         <v>250000</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B28" s="4">
         <v>5</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B29" s="4">
         <v>4</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B30" s="4">
         <v>60</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B31" s="4">
         <v>54</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B32" s="21">
         <f>B26/12</f>
         <v>8.3333333333333332E-3</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B33" s="4">
         <v>5</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B34" s="3">
         <v>3000</v>
@@ -1530,35 +1530,35 @@
         <v>21</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B35" s="6">
         <v>1</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B36" s="22">
         <v>8</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -4233,7 +4233,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="24" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -4256,49 +4256,49 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="F2" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -8309,7 +8309,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -8341,70 +8341,70 @@
     </row>
     <row r="2" spans="1:28" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="M2" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="M2" s="13" t="s">
+      <c r="O2" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="P2" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="S2" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="T2" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="P2" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="S2" s="13" t="s">
+      <c r="U2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="V2" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="W2" s="2"/>
       <c r="X2" s="2"/>
@@ -14080,7 +14080,7 @@
   <sheetData>
     <row r="1" spans="1:24" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="24" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C1" s="25"/>
       <c r="D1" s="25"/>
@@ -14095,73 +14095,73 @@
     </row>
     <row r="2" spans="1:24" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="J2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="M2" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="J2" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="L2" s="2" t="s">
+      <c r="N2" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="M2" s="16" t="s">
+      <c r="O2" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="N2" s="13" t="s">
+      <c r="P2" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q2" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="R2" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="P2" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q2" s="13" t="s">
+      <c r="S2" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="T2" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="R2" s="13" t="s">
+      <c r="U2" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="S2" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="T2" s="13" t="s">
+      <c r="V2" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="W2" s="13" t="s">
         <v>130</v>
-      </c>
-      <c r="U2" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="V2" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="W2" s="13" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
@@ -19707,7 +19707,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="24" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -19717,7 +19717,7 @@
     </row>
     <row r="2" spans="1:6" ht="28.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -19727,22 +19727,22 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>